<commit_message>
chore: sync excel data and deploy (2026-06-16 13:12)
</commit_message>
<xml_diff>
--- a/data/공모_260612.xlsx
+++ b/data/공모_260612.xlsx
@@ -623,22 +623,22 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>6,743</t>
+          <t>6,862</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>3,641</t>
+          <t>3,689</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>18,309</t>
+          <t>18,294</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -653,12 +653,12 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>50,308</t>
+          <t>50,279</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
-          <t>5,401</t>
+          <t>5,416</t>
         </is>
       </c>
       <c r="J6" s="10" t="inlineStr">
@@ -693,7 +693,7 @@
       </c>
       <c r="P6" s="10" t="inlineStr">
         <is>
-          <t>84,466</t>
+          <t>84,603</t>
         </is>
       </c>
       <c r="Q6" s="10" t="inlineStr">
@@ -703,12 +703,12 @@
       </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
-          <t>226</t>
+          <t>137</t>
         </is>
       </c>
       <c r="S6" s="10" t="inlineStr">
         <is>
-          <t>-16,106</t>
+          <t>-15,969</t>
         </is>
       </c>
     </row>
@@ -720,17 +720,17 @@
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>900</t>
+          <t>898</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>523</t>
+          <t>522</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>5,112</t>
+          <t>5,206</t>
         </is>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -750,7 +750,7 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>19,553</t>
+          <t>20,480</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="P7" s="10" t="inlineStr">
         <is>
-          <t>26,998</t>
+          <t>28,018</t>
         </is>
       </c>
       <c r="Q7" s="10" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="R7" s="10" t="inlineStr">
         <is>
-          <t>-69</t>
+          <t>1,020</t>
         </is>
       </c>
       <c r="S7" s="10" t="inlineStr">
         <is>
-          <t>-1,621</t>
+          <t>-601</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>4,065</t>
+          <t>4,165</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>405</t>
+          <t>404</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>24,381</t>
+          <t>25,166</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
@@ -857,7 +857,7 @@
       </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>53</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="P8" s="10" t="inlineStr">
         <is>
-          <t>30,785</t>
+          <t>31,668</t>
         </is>
       </c>
       <c r="Q8" s="10" t="inlineStr">
@@ -897,12 +897,12 @@
       </c>
       <c r="R8" s="10" t="inlineStr">
         <is>
-          <t>519</t>
+          <t>883</t>
         </is>
       </c>
       <c r="S8" s="10" t="inlineStr">
         <is>
-          <t>11,633</t>
+          <t>12,517</t>
         </is>
       </c>
     </row>
@@ -914,7 +914,7 @@
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>1,027</t>
+          <t>1,033</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
-          <t>1,027</t>
+          <t>1,033</t>
         </is>
       </c>
       <c r="Q9" s="10" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="S9" s="10" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>415</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1108,7 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>3,246</t>
+          <t>3,303</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>658</t>
+          <t>657</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>33,419</t>
+          <t>33,266</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="P11" s="10" t="inlineStr">
         <is>
-          <t>44,478</t>
+          <t>44,382</t>
         </is>
       </c>
       <c r="Q11" s="10" t="inlineStr">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>-96</t>
         </is>
       </c>
       <c r="S11" s="10" t="inlineStr">
         <is>
-          <t>4,523</t>
+          <t>4,426</t>
         </is>
       </c>
     </row>
@@ -1205,7 +1205,7 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>1,245</t>
+          <t>1,251</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
@@ -1275,7 +1275,7 @@
       </c>
       <c r="P12" s="10" t="inlineStr">
         <is>
-          <t>1,245</t>
+          <t>1,251</t>
         </is>
       </c>
       <c r="Q12" s="10" t="inlineStr">
@@ -1285,12 +1285,12 @@
       </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>7</t>
         </is>
       </c>
       <c r="S12" s="10" t="inlineStr">
         <is>
-          <t>408</t>
+          <t>415</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>7,398</t>
+          <t>7,491</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1312,12 +1312,12 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>3,273</t>
+          <t>3,259</t>
         </is>
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>18,486</t>
+          <t>18,683</t>
         </is>
       </c>
       <c r="F13" s="10" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
-          <t>540</t>
+          <t>538</t>
         </is>
       </c>
       <c r="J13" s="10" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="P13" s="10" t="inlineStr">
         <is>
-          <t>29,830</t>
+          <t>30,103</t>
         </is>
       </c>
       <c r="Q13" s="10" t="inlineStr">
@@ -1382,12 +1382,12 @@
       </c>
       <c r="R13" s="10" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>273</t>
         </is>
       </c>
       <c r="S13" s="10" t="inlineStr">
         <is>
-          <t>8,357</t>
+          <t>8,629</t>
         </is>
       </c>
     </row>
@@ -1496,22 +1496,22 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>558,325</t>
+          <t>588,459</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>9,905</t>
+          <t>9,912</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>12,534</t>
+          <t>12,539</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>110,748</t>
+          <t>110,315</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr">
@@ -1521,22 +1521,22 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>4,732</t>
+          <t>4,736</t>
         </is>
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>78,333</t>
+          <t>79,609</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>158,568</t>
+          <t>166,901</t>
         </is>
       </c>
       <c r="J15" s="10" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>599</t>
         </is>
       </c>
       <c r="K15" s="10" t="inlineStr">
@@ -1546,12 +1546,12 @@
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>13,016</t>
+          <t>13,274</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
         <is>
-          <t>15,316</t>
+          <t>16,988</t>
         </is>
       </c>
       <c r="N15" s="10" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
-          <t>962,087</t>
+          <t>1,003,331</t>
         </is>
       </c>
       <c r="Q15" s="10" t="inlineStr">
@@ -1576,12 +1576,12 @@
       </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
-          <t>1,445</t>
+          <t>41,244</t>
         </is>
       </c>
       <c r="S15" s="10" t="inlineStr">
         <is>
-          <t>380,822</t>
+          <t>422,066</t>
         </is>
       </c>
     </row>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>5,799</t>
+          <t>5,802</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
-          <t>6,648</t>
+          <t>6,651</t>
         </is>
       </c>
       <c r="Q17" s="10" t="inlineStr">
@@ -1770,12 +1770,12 @@
       </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="S17" s="10" t="inlineStr">
         <is>
-          <t>-258</t>
+          <t>-255</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>460</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="P18" s="10" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>460</t>
         </is>
       </c>
       <c r="Q18" s="10" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S18" s="10" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>1,738</t>
+          <t>1,789</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>2,135</t>
+          <t>2,137</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>2,346</t>
+          <t>2,339</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>32,005</t>
+          <t>32,491</t>
         </is>
       </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>206</t>
+          <t>215</t>
         </is>
       </c>
       <c r="J19" s="10" t="inlineStr">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="P19" s="10" t="inlineStr">
         <is>
-          <t>38,466</t>
+          <t>39,007</t>
         </is>
       </c>
       <c r="Q19" s="10" t="inlineStr">
@@ -1964,12 +1964,12 @@
       </c>
       <c r="R19" s="10" t="inlineStr">
         <is>
-          <t>1,159</t>
+          <t>541</t>
         </is>
       </c>
       <c r="S19" s="10" t="inlineStr">
         <is>
-          <t>14,873</t>
+          <t>15,414</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>4,918</t>
+          <t>4,920</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="P20" s="10" t="inlineStr">
         <is>
-          <t>4,918</t>
+          <t>4,920</t>
         </is>
       </c>
       <c r="Q20" s="10" t="inlineStr">
@@ -2061,12 +2061,12 @@
       </c>
       <c r="R20" s="10" t="inlineStr">
         <is>
-          <t>-17</t>
+          <t>2</t>
         </is>
       </c>
       <c r="S20" s="10" t="inlineStr">
         <is>
-          <t>-1,096</t>
+          <t>-1,094</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>214</t>
+          <t>213</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>2,302</t>
+          <t>2,344</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="P21" s="10" t="inlineStr">
         <is>
-          <t>2,757</t>
+          <t>2,799</t>
         </is>
       </c>
       <c r="Q21" s="10" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
-          <t>-2</t>
+          <t>42</t>
         </is>
       </c>
       <c r="S21" s="10" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>215</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>1,471</t>
+          <t>1,494</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -2185,12 +2185,12 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>418</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>1,820</t>
+          <t>2,876</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -2205,12 +2205,12 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>40,044</t>
+          <t>41,056</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>1,015</t>
+          <t>1,019</t>
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="P22" s="10" t="inlineStr">
         <is>
-          <t>44,802</t>
+          <t>46,888</t>
         </is>
       </c>
       <c r="Q22" s="10" t="inlineStr">
@@ -2255,12 +2255,12 @@
       </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
-          <t>-393</t>
+          <t>2,086</t>
         </is>
       </c>
       <c r="S22" s="10" t="inlineStr">
         <is>
-          <t>12,961</t>
+          <t>15,047</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t>21,079</t>
+          <t>21,450</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="P23" s="10" t="inlineStr">
         <is>
-          <t>21,079</t>
+          <t>21,450</t>
         </is>
       </c>
       <c r="Q23" s="10" t="inlineStr">
@@ -2352,12 +2352,12 @@
       </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
-          <t>723</t>
+          <t>370</t>
         </is>
       </c>
       <c r="S23" s="10" t="inlineStr">
         <is>
-          <t>11,144</t>
+          <t>11,514</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>779,964</t>
+          <t>816,929</t>
         </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
@@ -2379,12 +2379,12 @@
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>35,200</t>
+          <t>36,070</t>
         </is>
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>222,364</t>
+          <t>223,368</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
@@ -2394,22 +2394,22 @@
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>5,179</t>
+          <t>5,185</t>
         </is>
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>209,336</t>
+          <t>212,491</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>475,866</t>
+          <t>497,363</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr">
         <is>
-          <t>5,105</t>
+          <t>5,031</t>
         </is>
       </c>
       <c r="K24" s="10" t="inlineStr">
@@ -2424,7 +2424,7 @@
       </c>
       <c r="M24" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="N24" s="10" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="P24" s="10" t="inlineStr">
         <is>
-          <t>1,733,076</t>
+          <t>1,798,500</t>
         </is>
       </c>
       <c r="Q24" s="10" t="inlineStr">
@@ -2449,12 +2449,12 @@
       </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
-          <t>18,005</t>
+          <t>65,424</t>
         </is>
       </c>
       <c r="S24" s="10" t="inlineStr">
         <is>
-          <t>689,192</t>
+          <t>754,616</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>152</t>
+          <t>149</t>
         </is>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="P26" s="10" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>499</t>
         </is>
       </c>
       <c r="Q26" s="10" t="inlineStr">
@@ -2643,12 +2643,12 @@
       </c>
       <c r="R26" s="10" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="S26" s="10" t="inlineStr">
         <is>
-          <t>103</t>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t>17,769</t>
+          <t>17,764</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>894</t>
+          <t>897</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr">
@@ -2685,12 +2685,12 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>114</t>
         </is>
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>51,954</t>
+          <t>53,034</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="M27" s="10" t="inlineStr">
         <is>
-          <t>1,237</t>
+          <t>1,233</t>
         </is>
       </c>
       <c r="N27" s="10" t="inlineStr">
@@ -2730,7 +2730,7 @@
       </c>
       <c r="P27" s="10" t="inlineStr">
         <is>
-          <t>80,047</t>
+          <t>81,118</t>
         </is>
       </c>
       <c r="Q27" s="10" t="inlineStr">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="R27" s="10" t="inlineStr">
         <is>
-          <t>-496</t>
+          <t>1,071</t>
         </is>
       </c>
       <c r="S27" s="10" t="inlineStr">
         <is>
-          <t>23,538</t>
+          <t>24,609</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2757,7 @@
       </c>
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t>133,513</t>
+          <t>140,020</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
@@ -2767,12 +2767,12 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>8,093</t>
+          <t>8,111</t>
         </is>
       </c>
       <c r="E28" s="10" t="inlineStr">
         <is>
-          <t>59,748</t>
+          <t>59,955</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -2782,17 +2782,17 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>186</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>127,065</t>
+          <t>127,858</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>17,659</t>
+          <t>17,958</t>
         </is>
       </c>
       <c r="J28" s="10" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="P28" s="10" t="inlineStr">
         <is>
-          <t>347,311</t>
+          <t>355,134</t>
         </is>
       </c>
       <c r="Q28" s="10" t="inlineStr">
@@ -2837,12 +2837,12 @@
       </c>
       <c r="R28" s="10" t="inlineStr">
         <is>
-          <t>6,150</t>
+          <t>7,823</t>
         </is>
       </c>
       <c r="S28" s="10" t="inlineStr">
         <is>
-          <t>123,859</t>
+          <t>131,683</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t>4,370</t>
+          <t>4,428</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
@@ -2864,12 +2864,12 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>2,229</t>
+          <t>2,228</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>4,981</t>
+          <t>5,003</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr">
@@ -2879,17 +2879,17 @@
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>73</t>
         </is>
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>112,144</t>
+          <t>115,434</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>118</t>
         </is>
       </c>
       <c r="J29" s="10" t="inlineStr">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="P29" s="10" t="inlineStr">
         <is>
-          <t>123,949</t>
+          <t>127,319</t>
         </is>
       </c>
       <c r="Q29" s="10" t="inlineStr">
@@ -2934,12 +2934,12 @@
       </c>
       <c r="R29" s="10" t="inlineStr">
         <is>
-          <t>465</t>
+          <t>3,370</t>
         </is>
       </c>
       <c r="S29" s="10" t="inlineStr">
         <is>
-          <t>18,264</t>
+          <t>21,634</t>
         </is>
       </c>
     </row>
@@ -2951,7 +2951,7 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>1,545</t>
+          <t>1,599</t>
         </is>
       </c>
       <c r="C30" s="10" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>976</t>
+          <t>975</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -2981,12 +2981,12 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>15,721</t>
+          <t>15,516</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>143</t>
         </is>
       </c>
       <c r="J30" s="10" t="inlineStr">
@@ -3021,7 +3021,7 @@
       </c>
       <c r="P30" s="10" t="inlineStr">
         <is>
-          <t>19,442</t>
+          <t>19,291</t>
         </is>
       </c>
       <c r="Q30" s="10" t="inlineStr">
@@ -3031,12 +3031,12 @@
       </c>
       <c r="R30" s="10" t="inlineStr">
         <is>
-          <t>678</t>
+          <t>-151</t>
         </is>
       </c>
       <c r="S30" s="10" t="inlineStr">
         <is>
-          <t>-7,154</t>
+          <t>-7,305</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3145,7 @@
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>2,488</t>
+          <t>2,503</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>616</t>
+          <t>615</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="P32" s="10" t="inlineStr">
         <is>
-          <t>3,287</t>
+          <t>3,300</t>
         </is>
       </c>
       <c r="Q32" s="10" t="inlineStr">
@@ -3225,12 +3225,12 @@
       </c>
       <c r="R32" s="10" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>14</t>
         </is>
       </c>
       <c r="S32" s="10" t="inlineStr">
         <is>
-          <t>-183</t>
+          <t>-170</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="B33" s="10" t="inlineStr">
         <is>
-          <t>386</t>
+          <t>384</t>
         </is>
       </c>
       <c r="C33" s="10" t="inlineStr">
@@ -3312,7 +3312,7 @@
       </c>
       <c r="P33" s="10" t="inlineStr">
         <is>
-          <t>1,436</t>
+          <t>1,433</t>
         </is>
       </c>
       <c r="Q33" s="10" t="inlineStr">
@@ -3322,12 +3322,12 @@
       </c>
       <c r="R33" s="10" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="S33" s="10" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="B35" s="10" t="inlineStr">
         <is>
-          <t>79,748</t>
+          <t>83,073</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
@@ -3446,12 +3446,12 @@
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>4,184</t>
+          <t>4,209</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>10,627</t>
+          <t>10,594</t>
         </is>
       </c>
       <c r="F35" s="10" t="inlineStr">
@@ -3466,12 +3466,12 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>101,898</t>
+          <t>108,371</t>
         </is>
       </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
-          <t>16,756</t>
+          <t>16,865</t>
         </is>
       </c>
       <c r="J35" s="10" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="P35" s="10" t="inlineStr">
         <is>
-          <t>213,825</t>
+          <t>223,724</t>
         </is>
       </c>
       <c r="Q35" s="10" t="inlineStr">
@@ -3516,12 +3516,12 @@
       </c>
       <c r="R35" s="10" t="inlineStr">
         <is>
-          <t>-53</t>
+          <t>9,898</t>
         </is>
       </c>
       <c r="S35" s="10" t="inlineStr">
         <is>
-          <t>70,166</t>
+          <t>80,064</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>9,600</t>
+          <t>9,955</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>4,748</t>
+          <t>4,808</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
         <is>
-          <t>36,882</t>
+          <t>36,425</t>
         </is>
       </c>
       <c r="F36" s="10" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="H36" s="10" t="inlineStr">
         <is>
-          <t>170,295</t>
+          <t>171,510</t>
         </is>
       </c>
       <c r="I36" s="10" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="J36" s="10" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>93</t>
         </is>
       </c>
       <c r="K36" s="10" t="inlineStr">
@@ -3603,7 +3603,7 @@
       </c>
       <c r="P36" s="10" t="inlineStr">
         <is>
-          <t>221,801</t>
+          <t>222,972</t>
         </is>
       </c>
       <c r="Q36" s="10" t="inlineStr">
@@ -3613,12 +3613,12 @@
       </c>
       <c r="R36" s="10" t="inlineStr">
         <is>
-          <t>5,913</t>
+          <t>1,171</t>
         </is>
       </c>
       <c r="S36" s="10" t="inlineStr">
         <is>
-          <t>62,542</t>
+          <t>63,713</t>
         </is>
       </c>
     </row>
@@ -3630,7 +3630,7 @@
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>785</t>
+          <t>788</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
@@ -3640,7 +3640,7 @@
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>1,916</t>
+          <t>1,915</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="I37" s="10" t="inlineStr">
         <is>
-          <t>1,303</t>
+          <t>1,300</t>
         </is>
       </c>
       <c r="J37" s="10" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="P37" s="10" t="inlineStr">
         <is>
-          <t>9,723</t>
+          <t>9,721</t>
         </is>
       </c>
       <c r="Q37" s="10" t="inlineStr">
@@ -3710,12 +3710,12 @@
       </c>
       <c r="R37" s="10" t="inlineStr">
         <is>
-          <t>-302</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="S37" s="10" t="inlineStr">
         <is>
-          <t>3,500</t>
+          <t>3,498</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>779</t>
+          <t>807</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
@@ -3834,7 +3834,7 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>1,054</t>
+          <t>1,075</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
-          <t>583</t>
+          <t>584</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="P39" s="10" t="inlineStr">
         <is>
-          <t>4,502</t>
+          <t>4,553</t>
         </is>
       </c>
       <c r="Q39" s="10" t="inlineStr">
@@ -3904,12 +3904,12 @@
       </c>
       <c r="R39" s="10" t="inlineStr">
         <is>
-          <t>-25</t>
+          <t>51</t>
         </is>
       </c>
       <c r="S39" s="10" t="inlineStr">
         <is>
-          <t>1,449</t>
+          <t>1,500</t>
         </is>
       </c>
     </row>
@@ -3931,12 +3931,12 @@
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>2,144</t>
+          <t>2,143</t>
         </is>
       </c>
       <c r="E40" s="10" t="inlineStr">
         <is>
-          <t>14,413</t>
+          <t>14,423</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>13,440</t>
+          <t>13,937</t>
         </is>
       </c>
       <c r="I40" s="10" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="P40" s="10" t="inlineStr">
         <is>
-          <t>31,334</t>
+          <t>31,840</t>
         </is>
       </c>
       <c r="Q40" s="10" t="inlineStr">
@@ -4001,12 +4001,12 @@
       </c>
       <c r="R40" s="10" t="inlineStr">
         <is>
-          <t>-681</t>
+          <t>506</t>
         </is>
       </c>
       <c r="S40" s="10" t="inlineStr">
         <is>
-          <t>-10,788</t>
+          <t>-10,282</t>
         </is>
       </c>
     </row>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>706</t>
+          <t>703</t>
         </is>
       </c>
       <c r="C42" s="10" t="inlineStr">
@@ -4125,12 +4125,12 @@
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>843</t>
+          <t>842</t>
         </is>
       </c>
       <c r="E42" s="10" t="inlineStr">
         <is>
-          <t>6,321</t>
+          <t>6,435</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
@@ -4145,7 +4145,7 @@
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>2,543</t>
+          <t>2,544</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
@@ -4185,7 +4185,7 @@
       </c>
       <c r="P42" s="10" t="inlineStr">
         <is>
-          <t>10,434</t>
+          <t>10,546</t>
         </is>
       </c>
       <c r="Q42" s="10" t="inlineStr">
@@ -4195,12 +4195,12 @@
       </c>
       <c r="R42" s="10" t="inlineStr">
         <is>
-          <t>-14</t>
+          <t>112</t>
         </is>
       </c>
       <c r="S42" s="10" t="inlineStr">
         <is>
-          <t>786</t>
+          <t>898</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
       </c>
       <c r="R43" s="10" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="S43" s="10" t="inlineStr">
@@ -4309,22 +4309,22 @@
       </c>
       <c r="B44" s="10" t="inlineStr">
         <is>
-          <t>147,146</t>
+          <t>153,243</t>
         </is>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
-          <t>409</t>
+          <t>415</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>56,019</t>
+          <t>57,503</t>
         </is>
       </c>
       <c r="E44" s="10" t="inlineStr">
         <is>
-          <t>97,379</t>
+          <t>97,361</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
@@ -4334,17 +4334,17 @@
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>367</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
         <is>
-          <t>146,867</t>
+          <t>150,684</t>
         </is>
       </c>
       <c r="I44" s="10" t="inlineStr">
         <is>
-          <t>48,533</t>
+          <t>48,616</t>
         </is>
       </c>
       <c r="J44" s="10" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="M44" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2,000</t>
         </is>
       </c>
       <c r="N44" s="10" t="inlineStr">
@@ -4379,7 +4379,7 @@
       </c>
       <c r="P44" s="10" t="inlineStr">
         <is>
-          <t>509,097</t>
+          <t>522,444</t>
         </is>
       </c>
       <c r="Q44" s="10" t="inlineStr">
@@ -4389,12 +4389,12 @@
       </c>
       <c r="R44" s="10" t="inlineStr">
         <is>
-          <t>7,527</t>
+          <t>13,347</t>
         </is>
       </c>
       <c r="S44" s="10" t="inlineStr">
         <is>
-          <t>202,875</t>
+          <t>216,222</t>
         </is>
       </c>
     </row>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>7,153</t>
+          <t>7,155</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
@@ -4416,12 +4416,12 @@
       </c>
       <c r="D45" s="10" t="inlineStr">
         <is>
-          <t>4,010</t>
+          <t>4,380</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
         <is>
-          <t>1,787</t>
+          <t>2,755</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr">
@@ -4476,7 +4476,7 @@
       </c>
       <c r="P45" s="10" t="inlineStr">
         <is>
-          <t>13,220</t>
+          <t>14,560</t>
         </is>
       </c>
       <c r="Q45" s="10" t="inlineStr">
@@ -4486,12 +4486,12 @@
       </c>
       <c r="R45" s="10" t="inlineStr">
         <is>
-          <t>-22</t>
+          <t>1,340</t>
         </is>
       </c>
       <c r="S45" s="10" t="inlineStr">
         <is>
-          <t>-1,913</t>
+          <t>-573</t>
         </is>
       </c>
     </row>
@@ -4513,12 +4513,12 @@
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>3,798</t>
+          <t>3,789</t>
         </is>
       </c>
       <c r="E46" s="10" t="inlineStr">
         <is>
-          <t>17,659</t>
+          <t>17,572</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
@@ -4558,7 +4558,7 @@
       </c>
       <c r="M46" s="10" t="inlineStr">
         <is>
-          <t>8,585</t>
+          <t>8,464</t>
         </is>
       </c>
       <c r="N46" s="10" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="P46" s="10" t="inlineStr">
         <is>
-          <t>30,292</t>
+          <t>30,074</t>
         </is>
       </c>
       <c r="Q46" s="10" t="inlineStr">
@@ -4583,12 +4583,12 @@
       </c>
       <c r="R46" s="10" t="inlineStr">
         <is>
-          <t>-342</t>
+          <t>-218</t>
         </is>
       </c>
       <c r="S46" s="10" t="inlineStr">
         <is>
-          <t>4,509</t>
+          <t>4,291</t>
         </is>
       </c>
     </row>
@@ -4600,7 +4600,7 @@
       </c>
       <c r="B47" s="10" t="inlineStr">
         <is>
-          <t>35,965</t>
+          <t>37,568</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
@@ -4610,12 +4610,12 @@
       </c>
       <c r="D47" s="10" t="inlineStr">
         <is>
-          <t>2,687</t>
+          <t>2,731</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
         <is>
-          <t>35,018</t>
+          <t>34,744</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr">
@@ -4625,17 +4625,17 @@
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
-          <t>4,553</t>
+          <t>4,609</t>
         </is>
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>71,084</t>
+          <t>73,606</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>4,000</t>
+          <t>4,143</t>
         </is>
       </c>
       <c r="J47" s="10" t="inlineStr">
@@ -4670,7 +4670,7 @@
       </c>
       <c r="P47" s="10" t="inlineStr">
         <is>
-          <t>153,366</t>
+          <t>157,461</t>
         </is>
       </c>
       <c r="Q47" s="10" t="inlineStr">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="R47" s="10" t="inlineStr">
         <is>
-          <t>3,707</t>
+          <t>4,095</t>
         </is>
       </c>
       <c r="S47" s="10" t="inlineStr">
         <is>
-          <t>9,780</t>
+          <t>13,875</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4697,7 @@
       </c>
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>23,943</t>
+          <t>24,652</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
-          <t>9,234</t>
+          <t>9,316</t>
         </is>
       </c>
       <c r="H48" s="10" t="inlineStr">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="P48" s="10" t="inlineStr">
         <is>
-          <t>33,177</t>
+          <t>33,969</t>
         </is>
       </c>
       <c r="Q48" s="10" t="inlineStr">
@@ -4777,12 +4777,12 @@
       </c>
       <c r="R48" s="10" t="inlineStr">
         <is>
-          <t>382</t>
+          <t>792</t>
         </is>
       </c>
       <c r="S48" s="10" t="inlineStr">
         <is>
-          <t>18,759</t>
+          <t>19,551</t>
         </is>
       </c>
     </row>
@@ -4794,7 +4794,7 @@
       </c>
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>2,103</t>
+          <t>2,114</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>918</t>
+          <t>917</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="P49" s="10" t="inlineStr">
         <is>
-          <t>6,984</t>
+          <t>6,993</t>
         </is>
       </c>
       <c r="Q49" s="10" t="inlineStr">
@@ -4874,12 +4874,12 @@
       </c>
       <c r="R49" s="10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="S49" s="10" t="inlineStr">
         <is>
-          <t>-95</t>
+          <t>-85</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>52,942</t>
+          <t>53,352</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -4961,7 +4961,7 @@
       </c>
       <c r="P50" s="10" t="inlineStr">
         <is>
-          <t>53,619</t>
+          <t>54,030</t>
         </is>
       </c>
       <c r="Q50" s="10" t="inlineStr">
@@ -4971,12 +4971,12 @@
       </c>
       <c r="R50" s="10" t="inlineStr">
         <is>
-          <t>133</t>
+          <t>411</t>
         </is>
       </c>
       <c r="S50" s="10" t="inlineStr">
         <is>
-          <t>22,912</t>
+          <t>23,323</t>
         </is>
       </c>
     </row>
@@ -5182,7 +5182,7 @@
       </c>
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>16,119</t>
+          <t>16,728</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -5192,12 +5192,12 @@
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>3,325</t>
+          <t>3,408</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
         <is>
-          <t>30,113</t>
+          <t>29,986</t>
         </is>
       </c>
       <c r="F53" s="10" t="inlineStr">
@@ -5207,17 +5207,17 @@
       </c>
       <c r="G53" s="10" t="inlineStr">
         <is>
-          <t>1,524</t>
+          <t>1,573</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
         <is>
-          <t>119,267</t>
+          <t>121,921</t>
         </is>
       </c>
       <c r="I53" s="10" t="inlineStr">
         <is>
-          <t>2,743</t>
+          <t>2,792</t>
         </is>
       </c>
       <c r="J53" s="10" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="P53" s="10" t="inlineStr">
         <is>
-          <t>179,635</t>
+          <t>182,950</t>
         </is>
       </c>
       <c r="Q53" s="10" t="inlineStr">
@@ -5262,12 +5262,12 @@
       </c>
       <c r="R53" s="10" t="inlineStr">
         <is>
-          <t>1,420</t>
+          <t>3,315</t>
         </is>
       </c>
       <c r="S53" s="10" t="inlineStr">
         <is>
-          <t>37,047</t>
+          <t>40,362</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="B55" s="10" t="inlineStr">
         <is>
-          <t>8,573</t>
+          <t>8,574</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -5386,12 +5386,12 @@
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>7,689</t>
+          <t>7,693</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
         <is>
-          <t>412</t>
+          <t>411</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr">
@@ -5446,7 +5446,7 @@
       </c>
       <c r="P55" s="10" t="inlineStr">
         <is>
-          <t>21,314</t>
+          <t>21,317</t>
         </is>
       </c>
       <c r="Q55" s="10" t="inlineStr">
@@ -5456,12 +5456,12 @@
       </c>
       <c r="R55" s="10" t="inlineStr">
         <is>
-          <t>-14</t>
+          <t>4</t>
         </is>
       </c>
       <c r="S55" s="10" t="inlineStr">
         <is>
-          <t>1,215</t>
+          <t>1,218</t>
         </is>
       </c>
     </row>
@@ -5473,22 +5473,22 @@
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>64,393</t>
+          <t>67,199</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>2,996</t>
+          <t>2,995</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>6,776</t>
+          <t>6,763</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
         <is>
-          <t>53,683</t>
+          <t>53,394</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr">
@@ -5498,22 +5498,22 @@
       </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
-          <t>2,112</t>
+          <t>2,181</t>
         </is>
       </c>
       <c r="H56" s="10" t="inlineStr">
         <is>
-          <t>59,724</t>
+          <t>60,375</t>
         </is>
       </c>
       <c r="I56" s="10" t="inlineStr">
         <is>
-          <t>7,842</t>
+          <t>8,231</t>
         </is>
       </c>
       <c r="J56" s="10" t="inlineStr">
         <is>
-          <t>170</t>
+          <t>167</t>
         </is>
       </c>
       <c r="K56" s="10" t="inlineStr">
@@ -5523,7 +5523,7 @@
       </c>
       <c r="L56" s="10" t="inlineStr">
         <is>
-          <t>42,352</t>
+          <t>43,162</t>
         </is>
       </c>
       <c r="M56" s="10" t="inlineStr">
@@ -5543,7 +5543,7 @@
       </c>
       <c r="P56" s="10" t="inlineStr">
         <is>
-          <t>240,048</t>
+          <t>244,467</t>
         </is>
       </c>
       <c r="Q56" s="10" t="inlineStr">
@@ -5553,12 +5553,12 @@
       </c>
       <c r="R56" s="10" t="inlineStr">
         <is>
-          <t>1,941</t>
+          <t>4,418</t>
         </is>
       </c>
       <c r="S56" s="10" t="inlineStr">
         <is>
-          <t>51,329</t>
+          <t>55,747</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>73,794</t>
+          <t>76,235</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -5580,12 +5580,12 @@
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>843</t>
+          <t>842</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
         <is>
-          <t>27,205</t>
+          <t>26,971</t>
         </is>
       </c>
       <c r="F57" s="10" t="inlineStr">
@@ -5595,22 +5595,22 @@
       </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
-          <t>322</t>
+          <t>321</t>
         </is>
       </c>
       <c r="H57" s="10" t="inlineStr">
         <is>
-          <t>50,964</t>
+          <t>51,319</t>
         </is>
       </c>
       <c r="I57" s="10" t="inlineStr">
         <is>
-          <t>13,815</t>
+          <t>13,891</t>
         </is>
       </c>
       <c r="J57" s="10" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>74</t>
         </is>
       </c>
       <c r="K57" s="10" t="inlineStr">
@@ -5640,7 +5640,7 @@
       </c>
       <c r="P57" s="10" t="inlineStr">
         <is>
-          <t>167,321</t>
+          <t>169,956</t>
         </is>
       </c>
       <c r="Q57" s="10" t="inlineStr">
@@ -5650,12 +5650,12 @@
       </c>
       <c r="R57" s="10" t="inlineStr">
         <is>
-          <t>2,036</t>
+          <t>2,635</t>
         </is>
       </c>
       <c r="S57" s="10" t="inlineStr">
         <is>
-          <t>40,360</t>
+          <t>42,996</t>
         </is>
       </c>
     </row>
@@ -5672,12 +5672,12 @@
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>799</t>
+          <t>800</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>433</t>
+          <t>432</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
@@ -5692,12 +5692,12 @@
       </c>
       <c r="G58" s="10" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>17</t>
         </is>
       </c>
       <c r="H58" s="10" t="inlineStr">
         <is>
-          <t>21,717</t>
+          <t>24,188</t>
         </is>
       </c>
       <c r="I58" s="10" t="inlineStr">
@@ -5737,7 +5737,7 @@
       </c>
       <c r="P58" s="10" t="inlineStr">
         <is>
-          <t>24,771</t>
+          <t>27,241</t>
         </is>
       </c>
       <c r="Q58" s="10" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="R58" s="10" t="inlineStr">
         <is>
-          <t>265</t>
+          <t>2,470</t>
         </is>
       </c>
       <c r="S58" s="10" t="inlineStr">
         <is>
-          <t>4,726</t>
+          <t>7,196</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>2,513</t>
+          <t>2,689</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
@@ -5794,7 +5794,7 @@
       </c>
       <c r="H59" s="10" t="inlineStr">
         <is>
-          <t>15,955</t>
+          <t>16,094</t>
         </is>
       </c>
       <c r="I59" s="10" t="inlineStr">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="P59" s="10" t="inlineStr">
         <is>
-          <t>18,721</t>
+          <t>19,036</t>
         </is>
       </c>
       <c r="Q59" s="10" t="inlineStr">
@@ -5844,12 +5844,12 @@
       </c>
       <c r="R59" s="10" t="inlineStr">
         <is>
-          <t>-298</t>
+          <t>315</t>
         </is>
       </c>
       <c r="S59" s="10" t="inlineStr">
         <is>
-          <t>464</t>
+          <t>779</t>
         </is>
       </c>
     </row>
@@ -5861,7 +5861,7 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>1,827</t>
+          <t>1,868</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
@@ -5871,12 +5871,12 @@
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>2,205</t>
+          <t>2,203</t>
         </is>
       </c>
       <c r="E60" s="10" t="inlineStr">
         <is>
-          <t>20,121</t>
+          <t>20,139</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>14,156</t>
+          <t>13,811</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="P60" s="10" t="inlineStr">
         <is>
-          <t>43,889</t>
+          <t>43,600</t>
         </is>
       </c>
       <c r="Q60" s="10" t="inlineStr">
@@ -5941,12 +5941,12 @@
       </c>
       <c r="R60" s="10" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>-289</t>
         </is>
       </c>
       <c r="S60" s="10" t="inlineStr">
         <is>
-          <t>-6,224</t>
+          <t>-6,513</t>
         </is>
       </c>
     </row>
@@ -5958,22 +5958,22 @@
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>2,034,815</t>
+          <t>2,127,576</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>22,491</t>
+          <t>22,502</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
         <is>
-          <t>188,994</t>
+          <t>192,061</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
         <is>
-          <t>807,824</t>
+          <t>809,448</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
@@ -5983,22 +5983,22 @@
       </c>
       <c r="G61" s="10" t="inlineStr">
         <is>
-          <t>35,355</t>
+          <t>35,494</t>
         </is>
       </c>
       <c r="H61" s="10" t="inlineStr">
         <is>
-          <t>1,642,609</t>
+          <t>1,675,929</t>
         </is>
       </c>
       <c r="I61" s="10" t="inlineStr">
         <is>
-          <t>761,630</t>
+          <t>792,633</t>
         </is>
       </c>
       <c r="J61" s="10" t="inlineStr">
         <is>
-          <t>9,118</t>
+          <t>9,024</t>
         </is>
       </c>
       <c r="K61" s="10" t="inlineStr">
@@ -6008,12 +6008,12 @@
       </c>
       <c r="L61" s="10" t="inlineStr">
         <is>
-          <t>105,133</t>
+          <t>106,201</t>
         </is>
       </c>
       <c r="M61" s="10" t="inlineStr">
         <is>
-          <t>26,085</t>
+          <t>31,632</t>
         </is>
       </c>
       <c r="N61" s="10" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="P61" s="10" t="inlineStr">
         <is>
-          <t>5,634,414</t>
+          <t>5,802,858</t>
         </is>
       </c>
       <c r="Q61" s="10" t="inlineStr">
@@ -6038,12 +6038,12 @@
       </c>
       <c r="R61" s="10" t="inlineStr">
         <is>
-          <t>50,706</t>
+          <t>168,445</t>
         </is>
       </c>
       <c r="S61" s="10" t="inlineStr">
         <is>
-          <t>1,787,252</t>
+          <t>1,955,696</t>
         </is>
       </c>
     </row>
@@ -6055,22 +6055,22 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>2,034,815</t>
+          <t>2,127,576</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>22,491</t>
+          <t>22,502</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>188,994</t>
+          <t>192,061</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>807,824</t>
+          <t>809,448</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
@@ -6080,22 +6080,22 @@
       </c>
       <c r="G62" s="10" t="inlineStr">
         <is>
-          <t>35,355</t>
+          <t>35,494</t>
         </is>
       </c>
       <c r="H62" s="10" t="inlineStr">
         <is>
-          <t>1,642,609</t>
+          <t>1,675,929</t>
         </is>
       </c>
       <c r="I62" s="10" t="inlineStr">
         <is>
-          <t>761,630</t>
+          <t>792,633</t>
         </is>
       </c>
       <c r="J62" s="10" t="inlineStr">
         <is>
-          <t>9,118</t>
+          <t>9,024</t>
         </is>
       </c>
       <c r="K62" s="10" t="inlineStr">
@@ -6105,12 +6105,12 @@
       </c>
       <c r="L62" s="10" t="inlineStr">
         <is>
-          <t>105,133</t>
+          <t>106,201</t>
         </is>
       </c>
       <c r="M62" s="10" t="inlineStr">
         <is>
-          <t>26,085</t>
+          <t>31,632</t>
         </is>
       </c>
       <c r="N62" s="10" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="P62" s="10" t="inlineStr">
         <is>
-          <t>5,634,414</t>
+          <t>5,802,858</t>
         </is>
       </c>
       <c r="Q62" s="10" t="inlineStr">
@@ -6135,12 +6135,12 @@
       </c>
       <c r="R62" s="10" t="inlineStr">
         <is>
-          <t>50,706</t>
+          <t>168,445</t>
         </is>
       </c>
       <c r="S62" s="10" t="inlineStr">
         <is>
-          <t>1,787,252</t>
+          <t>1,955,696</t>
         </is>
       </c>
     </row>

</xml_diff>